<commit_message>
adding new imports to ClimOO-SDC2
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations/ClimOO Ontology vocabulary - List.xlsx
+++ b/ClimOO material/materials for implementations/ClimOO Ontology vocabulary - List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715DBAB1-FB88-EC4D-B3CC-45B045DE9E48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5B2BD3-0CDB-034E-BAC2-E6C7D5117291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42460" yWindow="1780" windowWidth="27640" windowHeight="16440" xr2:uid="{871EAFEC-93A1-F947-B348-9B49072C2753}"/>
+    <workbookView xWindow="31300" yWindow="2460" windowWidth="27640" windowHeight="16440" xr2:uid="{871EAFEC-93A1-F947-B348-9B49072C2753}"/>
   </bookViews>
   <sheets>
     <sheet name="ClimOO Vocabulary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1664" uniqueCount="837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1687" uniqueCount="848">
   <si>
     <t>entity</t>
   </si>
@@ -2547,13 +2547,46 @@
   </si>
   <si>
     <t>process of increase in atmospheric CO2 and CO2-equivalent concentration</t>
+  </si>
+  <si>
+    <t>laminar</t>
+  </si>
+  <si>
+    <t>p-block molecular entity</t>
+  </si>
+  <si>
+    <t>main group molecular entity</t>
+  </si>
+  <si>
+    <t>carbon group molecular entity</t>
+  </si>
+  <si>
+    <t>macronutrient</t>
+  </si>
+  <si>
+    <t>nonmetal atom</t>
+  </si>
+  <si>
+    <t>nitrogen atom</t>
+  </si>
+  <si>
+    <t>nutrient</t>
+  </si>
+  <si>
+    <t>pnictogen</t>
+  </si>
+  <si>
+    <t>carbon group element atom</t>
+  </si>
+  <si>
+    <t>atom</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2579,6 +2612,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -2594,7 +2633,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -2617,11 +2656,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2633,6 +2685,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -2967,7 +3023,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B6896C0-3354-CF47-84D5-E5D7BD388021}">
-  <dimension ref="A1:E833"/>
+  <dimension ref="A1:E845"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="75.6640625" style="4" bestFit="1" customWidth="1"/>
@@ -10431,6 +10487,7 @@
       <c r="B829" s="1" t="s">
         <v>831</v>
       </c>
+      <c r="C829" s="3"/>
     </row>
     <row r="830" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A830" s="6" t="s">
@@ -10439,6 +10496,7 @@
       <c r="B830" s="1" t="s">
         <v>831</v>
       </c>
+      <c r="C830" s="3"/>
     </row>
     <row r="831" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A831" s="6" t="s">
@@ -10447,6 +10505,7 @@
       <c r="B831" s="1" t="s">
         <v>831</v>
       </c>
+      <c r="C831" s="3"/>
     </row>
     <row r="832" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A832" s="6" t="s">
@@ -10455,13 +10514,119 @@
       <c r="B832" s="1" t="s">
         <v>831</v>
       </c>
-    </row>
-    <row r="833" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C832" s="3"/>
+    </row>
+    <row r="833" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A833" s="6" t="s">
         <v>836</v>
       </c>
-      <c r="B833" s="1" t="s">
+      <c r="B833" s="7" t="s">
         <v>831</v>
+      </c>
+      <c r="C833" s="8"/>
+    </row>
+    <row r="834" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A834" s="9" t="s">
+        <v>837</v>
+      </c>
+      <c r="B834" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C834" s="3"/>
+    </row>
+    <row r="835" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A835" s="1" t="s">
+        <v>838</v>
+      </c>
+      <c r="B835" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C835" s="3"/>
+    </row>
+    <row r="836" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A836" s="1" t="s">
+        <v>839</v>
+      </c>
+      <c r="B836" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C836" s="3"/>
+    </row>
+    <row r="837" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A837" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="B837" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C837" s="3"/>
+    </row>
+    <row r="838" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A838" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="B838" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C838" s="3"/>
+    </row>
+    <row r="839" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A839" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B839" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C839" s="3"/>
+    </row>
+    <row r="840" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A840" s="1" t="s">
+        <v>842</v>
+      </c>
+      <c r="B840" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C840" s="3"/>
+    </row>
+    <row r="841" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A841" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="B841" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C841" s="3"/>
+    </row>
+    <row r="842" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A842" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="B842" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C842" s="3"/>
+    </row>
+    <row r="843" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A843" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="B843" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C843" s="3"/>
+    </row>
+    <row r="844" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A844" s="1" t="s">
+        <v>846</v>
+      </c>
+      <c r="B844" s="10" t="s">
+        <v>808</v>
+      </c>
+      <c r="C844" s="3"/>
+    </row>
+    <row r="845" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A845" s="4" t="s">
+        <v>847</v>
       </c>
     </row>
   </sheetData>

</xml_diff>